<commit_message>
feat: add PacketStorm.tsx and FinalFrame.jsx minigames
</commit_message>
<xml_diff>
--- a/docs/Synapse_Garage_Inventory_Template.xlsx
+++ b/docs/Synapse_Garage_Inventory_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alex\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCE97954-7318-4612-9568-AEF349EEFB3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55566356-34EE-4EC9-B61A-B9F8AF421BD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="7845" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="7845" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PowerSupplies" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,6 @@
     <sheet name="Cables" sheetId="5" r:id="rId5"/>
     <sheet name="Cooling" sheetId="6" r:id="rId6"/>
     <sheet name="ComponentInteractions" sheetId="7" r:id="rId7"/>
-    <sheet name="MarketplaceRules" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -43,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="736" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="450">
   <si>
     <t>item_id</t>
   </si>
@@ -171,18 +170,6 @@
     <t>effect_value</t>
   </si>
   <si>
-    <t>performance_multiplier</t>
-  </si>
-  <si>
-    <t>market_value_multiplier</t>
-  </si>
-  <si>
-    <t>repairable</t>
-  </si>
-  <si>
-    <t>can_return_to_new</t>
-  </si>
-  <si>
     <t>psu_rustcore_350_rebuilt</t>
   </si>
   <si>
@@ -1231,6 +1218,180 @@
   </si>
   <si>
     <t>New RapidCell SSD gives fast data access for premium AetherFrame workloads.</t>
+  </si>
+  <si>
+    <t>cooling_dustfan_80mm_used</t>
+  </si>
+  <si>
+    <t>cooling_dustfan_80mm_rebuilt</t>
+  </si>
+  <si>
+    <t>cooling_dustfan_80mm_new</t>
+  </si>
+  <si>
+    <t>cooling_coolgrid_120mm_used</t>
+  </si>
+  <si>
+    <t>cooling_coolgrid_120mm_rebuilt</t>
+  </si>
+  <si>
+    <t>cooling_coolgrid_120mm_new</t>
+  </si>
+  <si>
+    <t>cooling_frostcore_dual_used</t>
+  </si>
+  <si>
+    <t>cooling_frostcore_dual_rebuilt</t>
+  </si>
+  <si>
+    <t>cooling_frostcore_dual_new</t>
+  </si>
+  <si>
+    <t>DustFan</t>
+  </si>
+  <si>
+    <t>CoolGrid</t>
+  </si>
+  <si>
+    <t>FrostCore</t>
+  </si>
+  <si>
+    <t>80mm</t>
+  </si>
+  <si>
+    <t>120mm</t>
+  </si>
+  <si>
+    <t>2x120mm</t>
+  </si>
+  <si>
+    <t>Basic Fan</t>
+  </si>
+  <si>
+    <t>Performance Fan</t>
+  </si>
+  <si>
+    <t>Dual Cooling</t>
+  </si>
+  <si>
+    <t>42 dB</t>
+  </si>
+  <si>
+    <t>+3% stability</t>
+  </si>
+  <si>
+    <t>+2°C under high load</t>
+  </si>
+  <si>
+    <t>/assets/dashboard/components/cooling/cooling_dustfan_80mm_used.png</t>
+  </si>
+  <si>
+    <t>Used DustFan 80mm basic cooling fan with missing blades, visible rust, and limited airflow.</t>
+  </si>
+  <si>
+    <t>-8°C</t>
+  </si>
+  <si>
+    <t>-11°C</t>
+  </si>
+  <si>
+    <t>-14°C</t>
+  </si>
+  <si>
+    <t>-13°C</t>
+  </si>
+  <si>
+    <t>-17°C</t>
+  </si>
+  <si>
+    <t>-22°C</t>
+  </si>
+  <si>
+    <t>36 dB</t>
+  </si>
+  <si>
+    <t>30 dB</t>
+  </si>
+  <si>
+    <t>40 dB</t>
+  </si>
+  <si>
+    <t>34 dB</t>
+  </si>
+  <si>
+    <t>28 dB</t>
+  </si>
+  <si>
+    <t>44 dB</t>
+  </si>
+  <si>
+    <t>+9% stability</t>
+  </si>
+  <si>
+    <t>+20% stability</t>
+  </si>
+  <si>
+    <t>-2% efficiency with high-end GPUs</t>
+  </si>
+  <si>
+    <t>Limited cooling for AetherFrame GPUs</t>
+  </si>
+  <si>
+    <t>/assets/dashboard/components/cooling/cooling_dustfan_80mm_rebuilt.png</t>
+  </si>
+  <si>
+    <t>Rebuilt DustFan 80mm cooling fan with restored blades, moderate wear, and improved airflow.</t>
+  </si>
+  <si>
+    <t>/assets/dashboard/components/cooling/cooling_dustfan_80mm_new.png</t>
+  </si>
+  <si>
+    <t>New DustFan 80mm basic cooling fan with clean casing, full lights, and warranty label.</t>
+  </si>
+  <si>
+    <t>+3°C when used with multiple GPUs</t>
+  </si>
+  <si>
+    <t>-2% efficiency with weak PSU</t>
+  </si>
+  <si>
+    <t>Requires stable power delivery</t>
+  </si>
+  <si>
+    <t>/assets/dashboard/components/cooling/cooling_coolgrid_120mm_used.png</t>
+  </si>
+  <si>
+    <t>/assets/dashboard/components/cooling/cooling_coolgrid_120mm_rebuilt.png</t>
+  </si>
+  <si>
+    <t>/assets/dashboard/components/cooling/cooling_coolgrid_120mm_new.png</t>
+  </si>
+  <si>
+    <t>Used CoolGrid 120mm performance fan with one missing blade, visible rust, and reduced light function.</t>
+  </si>
+  <si>
+    <t>Rebuilt CoolGrid 120mm cooling fan with reduced rust, restored structure, and 50% lights working.</t>
+  </si>
+  <si>
+    <t>New CoolGrid 120mm performance cooling fan with clean casing, full lights, and warranty label.</t>
+  </si>
+  <si>
+    <t>/assets/dashboard/components/cooling/cooling_frostcore_dual_used.png</t>
+  </si>
+  <si>
+    <t>/assets/dashboard/components/cooling/cooling_frostcore_dual_rebuilt.png</t>
+  </si>
+  <si>
+    <t>/assets/dashboard/components/cooling/cooling_frostcore_dual_new.png</t>
+  </si>
+  <si>
+    <t>Used FrostCore 2x120mm dual cooling module with medium rust, no active lights, and no warranty label.</t>
+  </si>
+  <si>
+    <t>Rebuilt FrostCore 2x120mm dual cooling module with no rust, restored casing, and 50% lights working.</t>
+  </si>
+  <si>
+    <t>New FrostCore 2x120mm premium dual cooling module with clean casing, full blue lights, and gold warranty label.</t>
   </si>
 </sst>
 </file>
@@ -1277,7 +1438,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1296,11 +1457,29 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="52">
+  <dxfs count="53">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -1557,55 +1736,55 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7A3EDF64-F1FF-4B05-8B27-ADF0DD73A065}" name="Tabela1" displayName="Tabela1" ref="A1:O30" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7A3EDF64-F1FF-4B05-8B27-ADF0DD73A065}" name="Tabela1" displayName="Tabela1" ref="A1:O30" totalsRowShown="0" headerRowDxfId="52" dataDxfId="51">
   <autoFilter ref="A1:O30" xr:uid="{7A3EDF64-F1FF-4B05-8B27-ADF0DD73A065}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{B97BE3F4-4816-4350-BE34-CE14110F9F1E}" name="item_id" dataDxfId="49"/>
-    <tableColumn id="2" xr3:uid="{9FDEE5CD-2B72-4620-ABA0-5FE5FBDA3D18}" name="brand" dataDxfId="48"/>
-    <tableColumn id="3" xr3:uid="{138C752B-F607-4D55-ADA6-AEA76E132FC3}" name="model" dataDxfId="47"/>
-    <tableColumn id="4" xr3:uid="{C097A2EE-A2E4-4C53-B055-A1174C9C825F}" name="condition" dataDxfId="46"/>
-    <tableColumn id="5" xr3:uid="{AE6DC481-F8D0-4F00-B931-EECC84EC4513}" name="power_w" dataDxfId="45"/>
-    <tableColumn id="6" xr3:uid="{B75EB86B-4DC1-46C6-B2AB-381D044C2ECB}" name="avg_consumption_w" dataDxfId="44"/>
-    <tableColumn id="7" xr3:uid="{42FD26FF-FC0A-4E21-A72A-F0A37F70E821}" name="temperature_c" dataDxfId="43"/>
-    <tableColumn id="8" xr3:uid="{522DE2E9-9834-4156-867F-276C203B0D77}" name="performance" dataDxfId="42"/>
-    <tableColumn id="9" xr3:uid="{D81B3410-2FDA-4ED8-AF78-4D3596B5E3D1}" name="stability" dataDxfId="41"/>
-    <tableColumn id="10" xr3:uid="{D79C0A7A-8AD4-4779-990C-62665B3DD0A5}" name="failure_risk" dataDxfId="40"/>
-    <tableColumn id="11" xr3:uid="{87386702-E285-4A13-AD75-970DE2C4A3E5}" name="price" dataDxfId="39"/>
-    <tableColumn id="12" xr3:uid="{739424DC-A568-4056-8BF5-9811F7CD39C7}" name="boost" dataDxfId="38"/>
-    <tableColumn id="13" xr3:uid="{69218A97-3065-4DE6-BB37-E3C0FA1D936A}" name="penalty" dataDxfId="37"/>
-    <tableColumn id="14" xr3:uid="{F753A896-6DAB-41A9-9A13-51E2E4D4250A}" name="image_path" dataDxfId="36"/>
-    <tableColumn id="15" xr3:uid="{02A7BA6E-BAA5-4066-A6E1-801A0D5B8754}" name="description" dataDxfId="35"/>
+    <tableColumn id="1" xr3:uid="{B97BE3F4-4816-4350-BE34-CE14110F9F1E}" name="item_id" dataDxfId="50"/>
+    <tableColumn id="2" xr3:uid="{9FDEE5CD-2B72-4620-ABA0-5FE5FBDA3D18}" name="brand" dataDxfId="49"/>
+    <tableColumn id="3" xr3:uid="{138C752B-F607-4D55-ADA6-AEA76E132FC3}" name="model" dataDxfId="48"/>
+    <tableColumn id="4" xr3:uid="{C097A2EE-A2E4-4C53-B055-A1174C9C825F}" name="condition" dataDxfId="47"/>
+    <tableColumn id="5" xr3:uid="{AE6DC481-F8D0-4F00-B931-EECC84EC4513}" name="power_w" dataDxfId="46"/>
+    <tableColumn id="6" xr3:uid="{B75EB86B-4DC1-46C6-B2AB-381D044C2ECB}" name="avg_consumption_w" dataDxfId="45"/>
+    <tableColumn id="7" xr3:uid="{42FD26FF-FC0A-4E21-A72A-F0A37F70E821}" name="temperature_c" dataDxfId="44"/>
+    <tableColumn id="8" xr3:uid="{522DE2E9-9834-4156-867F-276C203B0D77}" name="performance" dataDxfId="43"/>
+    <tableColumn id="9" xr3:uid="{D81B3410-2FDA-4ED8-AF78-4D3596B5E3D1}" name="stability" dataDxfId="42"/>
+    <tableColumn id="10" xr3:uid="{D79C0A7A-8AD4-4779-990C-62665B3DD0A5}" name="failure_risk" dataDxfId="41"/>
+    <tableColumn id="11" xr3:uid="{87386702-E285-4A13-AD75-970DE2C4A3E5}" name="price" dataDxfId="40"/>
+    <tableColumn id="12" xr3:uid="{739424DC-A568-4056-8BF5-9811F7CD39C7}" name="boost" dataDxfId="39"/>
+    <tableColumn id="13" xr3:uid="{69218A97-3065-4DE6-BB37-E3C0FA1D936A}" name="penalty" dataDxfId="38"/>
+    <tableColumn id="14" xr3:uid="{F753A896-6DAB-41A9-9A13-51E2E4D4250A}" name="image_path" dataDxfId="37"/>
+    <tableColumn id="15" xr3:uid="{02A7BA6E-BAA5-4066-A6E1-801A0D5B8754}" name="description" dataDxfId="36"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{5D6AE5CA-5B5F-4B80-8BFC-20A621EBF300}" name="Tabela6" displayName="Tabela6" ref="A1:O16" totalsRowShown="0" headerRowDxfId="2" dataDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{5D6AE5CA-5B5F-4B80-8BFC-20A621EBF300}" name="Tabela6" displayName="Tabela6" ref="A1:O16" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2">
   <autoFilter ref="A1:O16" xr:uid="{5D6AE5CA-5B5F-4B80-8BFC-20A621EBF300}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{55AD33DB-EEA7-4348-8BF1-14A52C977ABD}" name="item_id" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{BCDB483F-C4C8-4E89-8A2B-7C683494B6E3}" name="brand" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{E4727708-16F5-4DD5-8169-430543B0A41A}" name="model" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{1633DA9F-A074-4522-87B9-407D3140D269}" name="condition" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{65AFF02C-D0F2-4DFE-BFDE-934FC87B8352}" name="vram_gb" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{B1D2F7E6-D679-4BB8-9C2D-9BDA1B61C0E9}" name="power_consumption_w" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{FEF64AB8-A259-4294-BA70-625FBDFC1A66}" name="temperature_c" dataDxfId="11"/>
-    <tableColumn id="8" xr3:uid="{81AEE153-759C-467C-B434-453DE04A7D6E}" name="ai_output" dataDxfId="10"/>
-    <tableColumn id="9" xr3:uid="{158A24B6-1742-47EC-B01C-BE2E63DAB71A}" name="stability" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{C4269CD6-E97C-42ED-ABB3-3A43086442AF}" name="failure_risk" dataDxfId="8"/>
-    <tableColumn id="11" xr3:uid="{2037E293-DCE4-4A72-8D94-35BF068552ED}" name="price" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{81637B24-8D45-43D0-AD9A-204658C5B133}" name="boost" dataDxfId="6"/>
-    <tableColumn id="13" xr3:uid="{A507532C-EA2B-43E7-9D80-B50BE2F5B276}" name="penalty" dataDxfId="5"/>
-    <tableColumn id="14" xr3:uid="{8487049A-15A3-4BD3-BD47-2658FF9150F3}" name="image_path" dataDxfId="4"/>
-    <tableColumn id="15" xr3:uid="{EB833ACB-5F37-45EA-A655-20FCF6C007C2}" name="description" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{55AD33DB-EEA7-4348-8BF1-14A52C977ABD}" name="item_id" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{BCDB483F-C4C8-4E89-8A2B-7C683494B6E3}" name="brand" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{E4727708-16F5-4DD5-8169-430543B0A41A}" name="model" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{1633DA9F-A074-4522-87B9-407D3140D269}" name="condition" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{65AFF02C-D0F2-4DFE-BFDE-934FC87B8352}" name="vram_gb" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{B1D2F7E6-D679-4BB8-9C2D-9BDA1B61C0E9}" name="power_consumption_w" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{FEF64AB8-A259-4294-BA70-625FBDFC1A66}" name="temperature_c" dataDxfId="12"/>
+    <tableColumn id="8" xr3:uid="{81AEE153-759C-467C-B434-453DE04A7D6E}" name="ai_output" dataDxfId="11"/>
+    <tableColumn id="9" xr3:uid="{158A24B6-1742-47EC-B01C-BE2E63DAB71A}" name="stability" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{C4269CD6-E97C-42ED-ABB3-3A43086442AF}" name="failure_risk" dataDxfId="9"/>
+    <tableColumn id="11" xr3:uid="{2037E293-DCE4-4A72-8D94-35BF068552ED}" name="price" dataDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{81637B24-8D45-43D0-AD9A-204658C5B133}" name="boost" dataDxfId="7"/>
+    <tableColumn id="13" xr3:uid="{A507532C-EA2B-43E7-9D80-B50BE2F5B276}" name="penalty" dataDxfId="6"/>
+    <tableColumn id="14" xr3:uid="{8487049A-15A3-4BD3-BD47-2658FF9150F3}" name="image_path" dataDxfId="5"/>
+    <tableColumn id="15" xr3:uid="{EB833ACB-5F37-45EA-A655-20FCF6C007C2}" name="description" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{772E3ED4-9524-4682-A06D-0737E33395F3}" name="Tabela4" displayName="Tabela4" ref="A1:O14" totalsRowShown="0" headerRowDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{772E3ED4-9524-4682-A06D-0737E33395F3}" name="Tabela4" displayName="Tabela4" ref="A1:O14" totalsRowShown="0" headerRowDxfId="20">
   <autoFilter ref="A1:O14" xr:uid="{772E3ED4-9524-4682-A06D-0737E33395F3}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{BEECCB5E-2882-4823-9CAE-358B4F9F9AB3}" name="item_id"/>
@@ -1629,7 +1808,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{39AFF7C7-D365-42E2-A58C-98BAF78FC1CC}" name="Tabela5" displayName="Tabela5" ref="A1:O11" totalsRowShown="0" headerRowDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{39AFF7C7-D365-42E2-A58C-98BAF78FC1CC}" name="Tabela5" displayName="Tabela5" ref="A1:O11" totalsRowShown="0" headerRowDxfId="19">
   <autoFilter ref="A1:O11" xr:uid="{39AFF7C7-D365-42E2-A58C-98BAF78FC1CC}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{143D2358-942C-4B72-B32F-360224B001AA}" name="item_id"/>
@@ -1653,29 +1832,52 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{92FCF59B-E1E7-430F-BBF1-6EDD96CD3FAC}" name="Tabela2" displayName="Tabela2" ref="A1:M13" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{92FCF59B-E1E7-430F-BBF1-6EDD96CD3FAC}" name="Tabela2" displayName="Tabela2" ref="A1:M13" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
   <autoFilter ref="A1:M13" xr:uid="{92FCF59B-E1E7-430F-BBF1-6EDD96CD3FAC}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{49D608D5-90AD-4A2F-A527-C016388C2D32}" name="item_id" dataDxfId="32"/>
-    <tableColumn id="2" xr3:uid="{F0DAC06B-6F56-46DD-860C-A7FE050FEC5E}" name="brand" dataDxfId="31"/>
-    <tableColumn id="3" xr3:uid="{D6ADE88B-35AD-4AC0-A89E-CA51AFFB14C6}" name="model" dataDxfId="30"/>
-    <tableColumn id="4" xr3:uid="{2CE97618-6EBC-4C13-A6B3-5F76730A6BED}" name="condition" dataDxfId="29"/>
-    <tableColumn id="5" xr3:uid="{FDFF257E-C997-4A3F-B1B9-778A81798836}" name="cable_type" dataDxfId="28"/>
-    <tableColumn id="6" xr3:uid="{04385D70-037E-419F-B3A8-ACED85C88E47}" name="power_support" dataDxfId="27"/>
-    <tableColumn id="7" xr3:uid="{8F038EA6-2823-47B6-BB30-4FF31B02D89D}" name="stability_bonus" dataDxfId="26"/>
-    <tableColumn id="8" xr3:uid="{42BF8B26-AEB0-41B7-B52B-A27AD23A845F}" name="temperature_bonus" dataDxfId="25"/>
-    <tableColumn id="9" xr3:uid="{3A9076AB-5628-4A4F-AC66-7F757FABC4DA}" name="price" dataDxfId="24"/>
-    <tableColumn id="10" xr3:uid="{9A0A5C9E-8E3A-4076-ACE4-07A1614F1692}" name="boost" dataDxfId="23"/>
-    <tableColumn id="11" xr3:uid="{9771ACAE-19CF-47A7-9E65-24D5E77B230D}" name="penalty" dataDxfId="22"/>
-    <tableColumn id="12" xr3:uid="{B9F8062B-C215-4266-AC70-0CB108E4A3DE}" name="image_path" dataDxfId="21"/>
-    <tableColumn id="13" xr3:uid="{2F8DD4B3-EBE1-4C20-96C0-49B640D12514}" name="description" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{49D608D5-90AD-4A2F-A527-C016388C2D32}" name="item_id" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{F0DAC06B-6F56-46DD-860C-A7FE050FEC5E}" name="brand" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{D6ADE88B-35AD-4AC0-A89E-CA51AFFB14C6}" name="model" dataDxfId="31"/>
+    <tableColumn id="4" xr3:uid="{2CE97618-6EBC-4C13-A6B3-5F76730A6BED}" name="condition" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{FDFF257E-C997-4A3F-B1B9-778A81798836}" name="cable_type" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{04385D70-037E-419F-B3A8-ACED85C88E47}" name="power_support" dataDxfId="28"/>
+    <tableColumn id="7" xr3:uid="{8F038EA6-2823-47B6-BB30-4FF31B02D89D}" name="stability_bonus" dataDxfId="27"/>
+    <tableColumn id="8" xr3:uid="{42BF8B26-AEB0-41B7-B52B-A27AD23A845F}" name="temperature_bonus" dataDxfId="26"/>
+    <tableColumn id="9" xr3:uid="{3A9076AB-5628-4A4F-AC66-7F757FABC4DA}" name="price" dataDxfId="25"/>
+    <tableColumn id="10" xr3:uid="{9A0A5C9E-8E3A-4076-ACE4-07A1614F1692}" name="boost" dataDxfId="24"/>
+    <tableColumn id="11" xr3:uid="{9771ACAE-19CF-47A7-9E65-24D5E77B230D}" name="penalty" dataDxfId="23"/>
+    <tableColumn id="12" xr3:uid="{B9F8062B-C215-4266-AC70-0CB108E4A3DE}" name="image_path" dataDxfId="22"/>
+    <tableColumn id="13" xr3:uid="{2F8DD4B3-EBE1-4C20-96C0-49B640D12514}" name="description" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{FD6C0E84-3017-4803-8A77-5E09B2B49FB9}" name="Tabela7" displayName="Tabela7" ref="A1:E54" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{E33CE388-8E10-4858-8BB3-6D4CD826F4D4}" name="Tabela8" displayName="Tabela8" ref="A1:N11" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:N11" xr:uid="{E33CE388-8E10-4858-8BB3-6D4CD826F4D4}"/>
+  <tableColumns count="14">
+    <tableColumn id="1" xr3:uid="{CBAFF751-2B1C-49FF-BA84-4767A9F1F507}" name="item_id"/>
+    <tableColumn id="2" xr3:uid="{F7DA013A-7DEF-4A61-843E-95437086EACD}" name="brand"/>
+    <tableColumn id="3" xr3:uid="{64EB6A39-E04B-4E3C-A95D-00811BA25662}" name="model"/>
+    <tableColumn id="4" xr3:uid="{C5A4FDAE-AEA5-4EBF-BBFB-27434A55EF4F}" name="condition"/>
+    <tableColumn id="5" xr3:uid="{8B7045D4-E7B2-42CE-80E4-208C51BDB80F}" name="cooling_type"/>
+    <tableColumn id="6" xr3:uid="{2FEFD502-9C67-4723-9576-3D8FE79DFF39}" name="cooling_power"/>
+    <tableColumn id="7" xr3:uid="{DE5E27B5-D111-4E40-BDBD-E4925F6F99D5}" name="temperature_reduction"/>
+    <tableColumn id="8" xr3:uid="{8EA0DD81-4849-4C2F-BB8A-A48A3ACE46DA}" name="stability_bonus"/>
+    <tableColumn id="9" xr3:uid="{79CBD3DF-5806-4986-8AD4-44F68ED77482}" name="noise_level"/>
+    <tableColumn id="10" xr3:uid="{696EADEE-4AF7-4458-8422-F305AAB11158}" name="price"/>
+    <tableColumn id="11" xr3:uid="{96379A1F-F436-4D40-8B73-AE79D8232CE2}" name="boost"/>
+    <tableColumn id="12" xr3:uid="{3C06F5F6-8FCE-4B8B-A174-0A9C40943847}" name="penalty"/>
+    <tableColumn id="13" xr3:uid="{7DE3F82F-7C5B-4B10-BD40-24F7AAE94A58}" name="image_path"/>
+    <tableColumn id="14" xr3:uid="{51501A2D-4D83-4DA9-9438-303EDE985BB4}" name="description"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{FD6C0E84-3017-4803-8A77-5E09B2B49FB9}" name="Tabela7" displayName="Tabela7" ref="A1:E54" totalsRowShown="0" headerRowDxfId="1">
   <autoFilter ref="A1:E54" xr:uid="{FD6C0E84-3017-4803-8A77-5E09B2B49FB9}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{AD1CB2AB-A464-4A23-80F5-4497FC3C0E85}" name="item_a"/>
@@ -1971,6 +2173,26 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="3">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{78682A38-703D-4F38-BDC0-06D98251E40F}">
+  <we:reference id="wa200010215" version="2.0.0.0" store="pt-BR" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200010215" version="2.0.0.0" store="WA200010215" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O30"/>
@@ -2038,7 +2260,7 @@
         <v>16</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>17</v>
@@ -2074,21 +2296,21 @@
         <v>20</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E3" s="2">
         <v>350</v>
@@ -2112,30 +2334,30 @@
         <v>1900</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="M3" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="O3" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E4" s="2">
         <v>350</v>
@@ -2159,27 +2381,27 @@
         <v>3000</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>64</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>17</v>
@@ -2206,30 +2428,30 @@
         <v>1950</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="M5" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="O5" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="O5" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E6" s="2">
         <v>450</v>
@@ -2253,30 +2475,30 @@
         <v>2850</v>
       </c>
       <c r="L6" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="O6" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="M6" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="N6" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="O6" s="2" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E7" s="2">
         <v>450</v>
@@ -2300,27 +2522,27 @@
         <v>4300</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="M7" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="N7" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="N7" s="2" t="s">
-        <v>73</v>
-      </c>
       <c r="O7" s="2" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>74</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>78</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>17</v>
@@ -2347,30 +2569,30 @@
         <v>2800</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E9" s="2">
         <v>600</v>
@@ -2394,30 +2616,30 @@
         <v>4600</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E10" s="2">
         <v>600</v>
@@ -2441,16 +2663,16 @@
         <v>6800</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
@@ -2863,13 +3085,13 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>267</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>17</v>
@@ -2896,30 +3118,30 @@
         <v>3200</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>267</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E3" s="2">
         <v>2</v>
@@ -2943,30 +3165,30 @@
         <v>4800</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>267</v>
-      </c>
       <c r="D4" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E4" s="2">
         <v>2</v>
@@ -2990,27 +3212,27 @@
         <v>6800</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>17</v>
@@ -3037,30 +3259,30 @@
         <v>72000</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E6" s="2">
         <v>4</v>
@@ -3084,30 +3306,30 @@
         <v>9800</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E7" s="2">
         <v>4</v>
@@ -3131,27 +3353,27 @@
         <v>13500</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>17</v>
@@ -3178,30 +3400,30 @@
         <v>14500</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E9" s="2">
         <v>6</v>
@@ -3225,30 +3447,30 @@
         <v>19500</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E10" s="2">
         <v>6</v>
@@ -3272,27 +3494,27 @@
         <v>26000</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>17</v>
@@ -3319,30 +3541,30 @@
         <v>28000</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E12" s="2">
         <v>8</v>
@@ -3366,30 +3588,30 @@
         <v>38000</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>266</v>
-      </c>
       <c r="C13" s="2" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E13" s="2">
         <v>8</v>
@@ -3413,16 +3635,16 @@
         <v>52000</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
@@ -3546,13 +3768,13 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C2" t="s">
         <v>153</v>
-      </c>
-      <c r="B2" t="s">
-        <v>156</v>
-      </c>
-      <c r="C2" t="s">
-        <v>157</v>
       </c>
       <c r="D2" t="s">
         <v>17</v>
@@ -3561,7 +3783,7 @@
         <v>4</v>
       </c>
       <c r="F2" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="G2">
         <v>58</v>
@@ -3579,36 +3801,36 @@
         <v>900</v>
       </c>
       <c r="L2" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="M2" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N2" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="O2" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B3" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C3" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D3" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E3">
         <v>4</v>
       </c>
       <c r="F3" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="G3">
         <v>52</v>
@@ -3626,36 +3848,36 @@
         <v>1400</v>
       </c>
       <c r="L3" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="M3" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="N3" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="O3" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B4" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C4" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D4" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E4">
         <v>4</v>
       </c>
       <c r="F4" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="G4">
         <v>46</v>
@@ -3673,27 +3895,27 @@
         <v>2200</v>
       </c>
       <c r="L4" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="M4" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="N4" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="O4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="B5" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C5" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="D5" t="s">
         <v>17</v>
@@ -3702,7 +3924,7 @@
         <v>8</v>
       </c>
       <c r="F5" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="G5">
         <v>62</v>
@@ -3720,36 +3942,36 @@
         <v>2500</v>
       </c>
       <c r="L5" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="M5" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="N5" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="O5" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="B6" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C6" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="D6" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E6">
         <v>8</v>
       </c>
       <c r="F6" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="G6">
         <v>56</v>
@@ -3767,36 +3989,36 @@
         <v>3800</v>
       </c>
       <c r="L6" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="M6" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="N6" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="O6" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>156</v>
+      </c>
+      <c r="B7" t="s">
         <v>160</v>
       </c>
-      <c r="B7" t="s">
-        <v>164</v>
-      </c>
       <c r="C7" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="D7" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E7">
         <v>8</v>
       </c>
       <c r="F7" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="G7">
         <v>50</v>
@@ -3814,27 +4036,27 @@
         <v>5200</v>
       </c>
       <c r="L7" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="N7" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="O7" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B8" t="s">
         <v>161</v>
       </c>
-      <c r="B8" t="s">
-        <v>165</v>
-      </c>
       <c r="C8" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D8" t="s">
         <v>17</v>
@@ -3843,7 +4065,7 @@
         <v>16</v>
       </c>
       <c r="F8" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="G8">
         <v>68</v>
@@ -3861,36 +4083,36 @@
         <v>6500</v>
       </c>
       <c r="L8" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="M8" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="N8" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="O8" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B9" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C9" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E9">
         <v>16</v>
       </c>
       <c r="F9" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="G9">
         <v>60</v>
@@ -3908,36 +4130,36 @@
         <v>9000</v>
       </c>
       <c r="L9" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="M9" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="N9" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="O9" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>159</v>
+      </c>
+      <c r="B10" t="s">
+        <v>161</v>
+      </c>
+      <c r="C10" t="s">
         <v>163</v>
       </c>
-      <c r="B10" t="s">
-        <v>165</v>
-      </c>
-      <c r="C10" t="s">
-        <v>167</v>
-      </c>
       <c r="D10" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E10">
         <v>16</v>
       </c>
       <c r="F10" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="G10">
         <v>54</v>
@@ -3955,16 +4177,16 @@
         <v>12500</v>
       </c>
       <c r="L10" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="M10" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="N10" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="O10" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -4037,22 +4259,22 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B2" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="C2" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="D2" t="s">
         <v>17</v>
       </c>
       <c r="E2" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="F2" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="G2">
         <v>100</v>
@@ -4070,36 +4292,36 @@
         <v>1800</v>
       </c>
       <c r="L2" t="s">
+        <v>216</v>
+      </c>
+      <c r="M2" t="s">
+        <v>168</v>
+      </c>
+      <c r="N2" t="s">
         <v>220</v>
       </c>
-      <c r="M2" t="s">
-        <v>172</v>
-      </c>
-      <c r="N2" t="s">
-        <v>224</v>
-      </c>
       <c r="O2" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B3" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="C3" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="D3" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E3" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="F3" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="G3">
         <v>110</v>
@@ -4117,36 +4339,36 @@
         <v>2800</v>
       </c>
       <c r="L3" t="s">
+        <v>217</v>
+      </c>
+      <c r="M3" t="s">
+        <v>169</v>
+      </c>
+      <c r="N3" t="s">
         <v>221</v>
       </c>
-      <c r="M3" t="s">
-        <v>173</v>
-      </c>
-      <c r="N3" t="s">
-        <v>225</v>
-      </c>
       <c r="O3" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="B4" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="C4" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="D4" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="F4" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="G4">
         <v>120</v>
@@ -4164,36 +4386,36 @@
         <v>4200</v>
       </c>
       <c r="L4" t="s">
+        <v>218</v>
+      </c>
+      <c r="M4" t="s">
+        <v>219</v>
+      </c>
+      <c r="N4" t="s">
         <v>222</v>
       </c>
-      <c r="M4" t="s">
-        <v>223</v>
-      </c>
-      <c r="N4" t="s">
-        <v>226</v>
-      </c>
       <c r="O4" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="B5" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="C5" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="D5" t="s">
         <v>17</v>
       </c>
       <c r="E5" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="F5" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="G5">
         <v>150</v>
@@ -4211,36 +4433,36 @@
         <v>4500</v>
       </c>
       <c r="L5" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="M5" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="N5" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="O5" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="B6" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="C6" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="D6" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E6" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="F6" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="G6">
         <v>170</v>
@@ -4258,36 +4480,36 @@
         <v>6200</v>
       </c>
       <c r="L6" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="M6" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="N6" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="O6" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="B7" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="C7" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="D7" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E7" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="F7" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="G7">
         <v>190</v>
@@ -4305,36 +4527,36 @@
         <v>8500</v>
       </c>
       <c r="L7" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="M7" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="N7" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="O7" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="B8" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="C8" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="D8" t="s">
         <v>17</v>
       </c>
       <c r="E8" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="F8" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="G8">
         <v>280</v>
@@ -4352,36 +4574,36 @@
         <v>7000</v>
       </c>
       <c r="L8" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="M8" s="7" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="N8" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="O8" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>207</v>
+      </c>
+      <c r="B9" t="s">
         <v>211</v>
       </c>
-      <c r="B9" t="s">
-        <v>215</v>
-      </c>
       <c r="C9" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="D9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E9" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="F9" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="G9">
         <v>320</v>
@@ -4399,36 +4621,36 @@
         <v>9800</v>
       </c>
       <c r="L9" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="M9" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="N9" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="O9" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="B10" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="C10" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="D10" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E10" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="F10" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="G10">
         <v>360</v>
@@ -4446,16 +4668,16 @@
         <v>13500</v>
       </c>
       <c r="L10" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="M10" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="N10" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="O10" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
     </row>
   </sheetData>
@@ -4529,371 +4751,371 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>17</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="G2" s="2">
         <v>3</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="I2" s="2">
         <v>600</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>104</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="G3" s="2">
         <v>6</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="I3" s="2">
         <v>1000</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>104</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="G4" s="2">
         <v>9</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="I4" s="2">
         <v>1500</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>17</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="G5" s="2">
         <v>6</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="I5" s="2">
         <v>1200</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>105</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>109</v>
       </c>
       <c r="G6" s="2">
         <v>9</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="I6" s="2">
         <v>1900</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>102</v>
-      </c>
       <c r="C7" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>105</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>109</v>
       </c>
       <c r="G7" s="2">
         <v>12</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="I7" s="2">
         <v>2800</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>103</v>
-      </c>
       <c r="C8" s="2" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>17</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G8" s="2">
         <v>9</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="I8" s="2">
         <v>2200</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>110</v>
       </c>
       <c r="G9" s="2">
         <v>13</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="I9" s="2">
         <v>3400</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>110</v>
       </c>
       <c r="G10" s="2">
         <v>16</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="I10" s="2">
         <v>4800</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -4951,10 +5173,14 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="14" width="28" customWidth="1"/>
+    <col min="1" max="1" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="11" width="28" customWidth="1"/>
+    <col min="12" max="12" width="35.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="69.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="104.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -5001,8 +5227,407 @@
         <v>14</v>
       </c>
     </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>392</v>
+      </c>
+      <c r="B2" t="s">
+        <v>401</v>
+      </c>
+      <c r="C2" t="s">
+        <v>404</v>
+      </c>
+      <c r="D2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" t="s">
+        <v>407</v>
+      </c>
+      <c r="F2">
+        <v>24</v>
+      </c>
+      <c r="G2" t="s">
+        <v>109</v>
+      </c>
+      <c r="H2" s="8">
+        <v>0.03</v>
+      </c>
+      <c r="I2" t="s">
+        <v>410</v>
+      </c>
+      <c r="J2">
+        <v>1200</v>
+      </c>
+      <c r="K2" t="s">
+        <v>411</v>
+      </c>
+      <c r="L2" t="s">
+        <v>412</v>
+      </c>
+      <c r="M2" t="s">
+        <v>413</v>
+      </c>
+      <c r="N2" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>393</v>
+      </c>
+      <c r="B3" t="s">
+        <v>401</v>
+      </c>
+      <c r="C3" t="s">
+        <v>404</v>
+      </c>
+      <c r="D3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E3" t="s">
+        <v>407</v>
+      </c>
+      <c r="F3">
+        <v>30</v>
+      </c>
+      <c r="G3" t="s">
+        <v>111</v>
+      </c>
+      <c r="H3" s="8">
+        <v>0.05</v>
+      </c>
+      <c r="I3" t="s">
+        <v>421</v>
+      </c>
+      <c r="J3">
+        <v>2200</v>
+      </c>
+      <c r="K3" t="s">
+        <v>329</v>
+      </c>
+      <c r="L3" t="s">
+        <v>429</v>
+      </c>
+      <c r="M3" t="s">
+        <v>431</v>
+      </c>
+      <c r="N3" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>394</v>
+      </c>
+      <c r="B4" t="s">
+        <v>401</v>
+      </c>
+      <c r="C4" t="s">
+        <v>404</v>
+      </c>
+      <c r="D4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E4" t="s">
+        <v>407</v>
+      </c>
+      <c r="F4">
+        <v>36</v>
+      </c>
+      <c r="G4" t="s">
+        <v>112</v>
+      </c>
+      <c r="H4" s="8">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="I4" t="s">
+        <v>422</v>
+      </c>
+      <c r="J4">
+        <v>3500</v>
+      </c>
+      <c r="K4" t="s">
+        <v>330</v>
+      </c>
+      <c r="L4" t="s">
+        <v>430</v>
+      </c>
+      <c r="M4" t="s">
+        <v>433</v>
+      </c>
+      <c r="N4" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>395</v>
+      </c>
+      <c r="B5" t="s">
+        <v>402</v>
+      </c>
+      <c r="C5" t="s">
+        <v>405</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" t="s">
+        <v>408</v>
+      </c>
+      <c r="F5">
+        <v>42</v>
+      </c>
+      <c r="G5" t="s">
+        <v>415</v>
+      </c>
+      <c r="H5" s="8">
+        <v>0.06</v>
+      </c>
+      <c r="I5" t="s">
+        <v>423</v>
+      </c>
+      <c r="J5">
+        <v>4200</v>
+      </c>
+      <c r="K5" t="s">
+        <v>344</v>
+      </c>
+      <c r="L5" t="s">
+        <v>435</v>
+      </c>
+      <c r="M5" t="s">
+        <v>438</v>
+      </c>
+      <c r="N5" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>396</v>
+      </c>
+      <c r="B6" t="s">
+        <v>402</v>
+      </c>
+      <c r="C6" t="s">
+        <v>405</v>
+      </c>
+      <c r="D6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" t="s">
+        <v>408</v>
+      </c>
+      <c r="F6">
+        <v>52</v>
+      </c>
+      <c r="G6" t="s">
+        <v>416</v>
+      </c>
+      <c r="H6" s="8">
+        <v>0.09</v>
+      </c>
+      <c r="I6" t="s">
+        <v>424</v>
+      </c>
+      <c r="J6">
+        <v>6200</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>427</v>
+      </c>
+      <c r="L6" t="s">
+        <v>436</v>
+      </c>
+      <c r="M6" t="s">
+        <v>439</v>
+      </c>
+      <c r="N6" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>397</v>
+      </c>
+      <c r="B7" t="s">
+        <v>402</v>
+      </c>
+      <c r="C7" t="s">
+        <v>405</v>
+      </c>
+      <c r="D7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" t="s">
+        <v>408</v>
+      </c>
+      <c r="F7">
+        <v>62</v>
+      </c>
+      <c r="G7" t="s">
+        <v>417</v>
+      </c>
+      <c r="H7" s="8">
+        <v>0.12</v>
+      </c>
+      <c r="I7" t="s">
+        <v>425</v>
+      </c>
+      <c r="J7">
+        <v>8500</v>
+      </c>
+      <c r="K7" t="s">
+        <v>347</v>
+      </c>
+      <c r="L7" t="s">
+        <v>437</v>
+      </c>
+      <c r="M7" t="s">
+        <v>440</v>
+      </c>
+      <c r="N7" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>398</v>
+      </c>
+      <c r="B8" t="s">
+        <v>403</v>
+      </c>
+      <c r="C8" t="s">
+        <v>406</v>
+      </c>
+      <c r="D8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" t="s">
+        <v>409</v>
+      </c>
+      <c r="F8">
+        <v>70</v>
+      </c>
+      <c r="G8" t="s">
+        <v>418</v>
+      </c>
+      <c r="H8" s="8">
+        <v>0.1</v>
+      </c>
+      <c r="I8" t="s">
+        <v>426</v>
+      </c>
+      <c r="J8">
+        <v>9500</v>
+      </c>
+      <c r="K8" t="s">
+        <v>331</v>
+      </c>
+      <c r="L8" t="s">
+        <v>331</v>
+      </c>
+      <c r="M8" t="s">
+        <v>444</v>
+      </c>
+      <c r="N8" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>399</v>
+      </c>
+      <c r="B9" t="s">
+        <v>403</v>
+      </c>
+      <c r="C9" t="s">
+        <v>406</v>
+      </c>
+      <c r="D9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" t="s">
+        <v>409</v>
+      </c>
+      <c r="F9">
+        <v>82</v>
+      </c>
+      <c r="G9" t="s">
+        <v>419</v>
+      </c>
+      <c r="H9" s="8">
+        <v>0.15</v>
+      </c>
+      <c r="I9" t="s">
+        <v>421</v>
+      </c>
+      <c r="J9">
+        <v>13500</v>
+      </c>
+      <c r="K9" t="s">
+        <v>350</v>
+      </c>
+      <c r="L9" t="s">
+        <v>350</v>
+      </c>
+      <c r="M9" t="s">
+        <v>445</v>
+      </c>
+      <c r="N9" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>400</v>
+      </c>
+      <c r="B10" t="s">
+        <v>403</v>
+      </c>
+      <c r="C10" t="s">
+        <v>406</v>
+      </c>
+      <c r="D10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E10" t="s">
+        <v>409</v>
+      </c>
+      <c r="F10">
+        <v>96</v>
+      </c>
+      <c r="G10" t="s">
+        <v>420</v>
+      </c>
+      <c r="H10" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="I10" t="s">
+        <v>422</v>
+      </c>
+      <c r="J10">
+        <v>19000</v>
+      </c>
+      <c r="K10" t="s">
+        <v>428</v>
+      </c>
+      <c r="L10" t="s">
+        <v>428</v>
+      </c>
+      <c r="M10" t="s">
+        <v>446</v>
+      </c>
+      <c r="N10" t="s">
+        <v>449</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -5037,682 +5662,682 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="B2" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C2" t="s">
         <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="E2" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="B3" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="C3" t="s">
         <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="E3" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="B4" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C4" t="s">
         <v>11</v>
       </c>
       <c r="D4" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="E4" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="B5" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="C5" t="s">
         <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="E5" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="B6" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C6" t="s">
         <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="E6" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="B7" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C7" t="s">
         <v>11</v>
       </c>
       <c r="D7" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="E7" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="B8" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C8" t="s">
         <v>11</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="E8" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="B9" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C9" t="s">
         <v>11</v>
       </c>
       <c r="D9" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="E9" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="B10" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C10" t="s">
         <v>11</v>
       </c>
       <c r="D10" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="E10" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B11" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="C11" t="s">
         <v>11</v>
       </c>
       <c r="D11" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="E11" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B12" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="C12" t="s">
         <v>11</v>
       </c>
       <c r="D12" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="E12" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B13" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="C13" t="s">
         <v>11</v>
       </c>
       <c r="D13" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="E13" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="B14" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="C14" t="s">
         <v>11</v>
       </c>
       <c r="D14" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="E14" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="B15" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="C15" t="s">
         <v>11</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="E15" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B16" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="C16" t="s">
         <v>11</v>
       </c>
       <c r="D16" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="E16" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="B17" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="C17" t="s">
         <v>11</v>
       </c>
       <c r="D17" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="E17" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B18" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="C18" t="s">
         <v>11</v>
       </c>
       <c r="D18" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="E18" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B19" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="C19" t="s">
         <v>11</v>
       </c>
       <c r="D19" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="E19" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="B20" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="C20" t="s">
         <v>11</v>
       </c>
       <c r="D20" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="E20" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B21" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="C21" t="s">
         <v>11</v>
       </c>
       <c r="D21" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="E21" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B22" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="C22" t="s">
         <v>11</v>
       </c>
       <c r="D22" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="E22" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="B23" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="C23" t="s">
         <v>12</v>
       </c>
       <c r="D23" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="E23" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="B24" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="C24" t="s">
         <v>12</v>
       </c>
       <c r="D24" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="E24" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="B25" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="C25" t="s">
         <v>11</v>
       </c>
       <c r="D25" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="E25" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="B26" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="C26" t="s">
         <v>11</v>
       </c>
       <c r="D26" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="E26" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="B27" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="C27" t="s">
         <v>12</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="E27" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="B28" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="C28" t="s">
         <v>11</v>
       </c>
       <c r="D28" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="E28" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="B29" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="C29" t="s">
         <v>11</v>
       </c>
       <c r="D29" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
       <c r="E29" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="B30" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="C30" t="s">
         <v>12</v>
       </c>
       <c r="D30" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
       <c r="E30" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="B31" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="C31" t="s">
         <v>11</v>
       </c>
       <c r="D31" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
       <c r="E31" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="B32" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="C32" t="s">
         <v>11</v>
       </c>
       <c r="D32" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
       <c r="E32" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="B33" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="C33" t="s">
         <v>12</v>
       </c>
       <c r="D33" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="E33" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="B34" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="C34" t="s">
         <v>12</v>
       </c>
       <c r="D34" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
       <c r="E34" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="B35" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="C35" t="s">
         <v>11</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
       <c r="E35" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="B36" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="C36" t="s">
         <v>11</v>
       </c>
       <c r="D36" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="E36" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B37" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="C37" t="s">
         <v>12</v>
       </c>
       <c r="D37" t="s">
-        <v>355</v>
+        <v>351</v>
       </c>
       <c r="E37" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="B38" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="C38" t="s">
         <v>11</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="E38" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="B39" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="C39" t="s">
         <v>11</v>
       </c>
       <c r="D39" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="E39" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="B40" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="C40" t="s">
         <v>11</v>
       </c>
       <c r="D40" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="E40" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="B41" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="C41" t="s">
         <v>11</v>
       </c>
       <c r="D41" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="E41" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
     </row>
   </sheetData>
@@ -5721,37 +6346,4 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="6" width="28" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>